<commit_message>
fixed typo in qrf_spatial_extents_updates.xlsx
</commit_message>
<xml_diff>
--- a/data/qrf_spatial_extents_updates.xlsx
+++ b/data/qrf_spatial_extents_updates.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\SnakeRiverFishHabitat\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DABD4CA3-3F89-473C-A8A3-A35F212A9357}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42CCA637-9A53-4E44-A711-2181F2C1D7DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="57480" yWindow="-120" windowWidth="16440" windowHeight="28320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7558" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7558" uniqueCount="66">
   <si>
     <t>unique_id</t>
   </si>
@@ -228,9 +228,6 @@
   </si>
   <si>
     <t>updated by Mike Ackerman on August 12, 2025 based on observed redds (IFWIS); sthd updated by Mike Ackerman on March 4, 2026 based of juvenile observations (FDAT)</t>
-  </si>
-  <si>
-    <t>Spawning and Rearing</t>
   </si>
   <si>
     <t>updated by Mike Ackerman on March 4, 2026 based on juvenile observations (FDAT)</t>
@@ -7269,10 +7266,10 @@
         <v>1</v>
       </c>
       <c r="F395" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G395" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G395" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="396" spans="1:7" x14ac:dyDescent="0.3">
@@ -7286,10 +7283,10 @@
         <v>1</v>
       </c>
       <c r="F396" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G396" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G396" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="397" spans="1:7" x14ac:dyDescent="0.3">
@@ -7354,10 +7351,10 @@
         <v>1</v>
       </c>
       <c r="F400" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G400" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G400" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="401" spans="1:7" x14ac:dyDescent="0.3">
@@ -7439,10 +7436,10 @@
         <v>1</v>
       </c>
       <c r="F405" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G405" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G405" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="406" spans="1:7" x14ac:dyDescent="0.3">
@@ -7507,10 +7504,10 @@
         <v>1</v>
       </c>
       <c r="F409" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G409" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G409" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="410" spans="1:7" x14ac:dyDescent="0.3">
@@ -7626,10 +7623,10 @@
         <v>1</v>
       </c>
       <c r="F416" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G416" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G416" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="417" spans="1:7" x14ac:dyDescent="0.3">
@@ -7745,10 +7742,10 @@
         <v>1</v>
       </c>
       <c r="F423" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G423" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G423" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="424" spans="1:7" x14ac:dyDescent="0.3">
@@ -7836,10 +7833,10 @@
         <v>1</v>
       </c>
       <c r="F428" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G428" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G428" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="429" spans="1:7" x14ac:dyDescent="0.3">
@@ -7853,10 +7850,10 @@
         <v>1</v>
       </c>
       <c r="F429" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G429" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G429" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="430" spans="1:7" x14ac:dyDescent="0.3">
@@ -7921,10 +7918,10 @@
         <v>1</v>
       </c>
       <c r="F433" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G433" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G433" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="434" spans="1:7" x14ac:dyDescent="0.3">
@@ -7955,10 +7952,10 @@
         <v>1</v>
       </c>
       <c r="F435" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G435" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G435" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="436" spans="1:7" x14ac:dyDescent="0.3">
@@ -7989,10 +7986,10 @@
         <v>1</v>
       </c>
       <c r="F437" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G437" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G437" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="438" spans="1:7" x14ac:dyDescent="0.3">
@@ -8057,10 +8054,10 @@
         <v>1</v>
       </c>
       <c r="F441" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G441" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G441" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="442" spans="1:7" x14ac:dyDescent="0.3">
@@ -8193,10 +8190,10 @@
         <v>1</v>
       </c>
       <c r="F449" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G449" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G449" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="450" spans="1:7" x14ac:dyDescent="0.3">
@@ -8573,10 +8570,10 @@
         <v>1</v>
       </c>
       <c r="F471" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G471" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G471" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="472" spans="1:7" x14ac:dyDescent="0.3">
@@ -8624,10 +8621,10 @@
         <v>1</v>
       </c>
       <c r="F474" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G474" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G474" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="475" spans="1:7" x14ac:dyDescent="0.3">
@@ -8692,10 +8689,10 @@
         <v>1</v>
       </c>
       <c r="F478" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G478" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G478" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="479" spans="1:7" x14ac:dyDescent="0.3">
@@ -8817,10 +8814,10 @@
         <v>1</v>
       </c>
       <c r="F485" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G485" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G485" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="486" spans="1:7" x14ac:dyDescent="0.3">
@@ -8851,10 +8848,10 @@
         <v>1</v>
       </c>
       <c r="F487" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G487" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G487" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="488" spans="1:7" x14ac:dyDescent="0.3">
@@ -8885,10 +8882,10 @@
         <v>1</v>
       </c>
       <c r="F489" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G489" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G489" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="490" spans="1:7" x14ac:dyDescent="0.3">
@@ -8902,10 +8899,10 @@
         <v>1</v>
       </c>
       <c r="F490" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G490" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G490" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="491" spans="1:7" x14ac:dyDescent="0.3">
@@ -9180,10 +9177,10 @@
         <v>1</v>
       </c>
       <c r="F506" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G506" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G506" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="507" spans="1:7" x14ac:dyDescent="0.3">
@@ -9288,10 +9285,10 @@
         <v>1</v>
       </c>
       <c r="F512" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G512" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G512" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="513" spans="1:7" x14ac:dyDescent="0.3">
@@ -9305,10 +9302,10 @@
         <v>1</v>
       </c>
       <c r="F513" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G513" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G513" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="514" spans="1:7" x14ac:dyDescent="0.3">
@@ -9532,10 +9529,10 @@
         <v>1</v>
       </c>
       <c r="F526" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G526" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G526" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="527" spans="1:7" x14ac:dyDescent="0.3">
@@ -9963,10 +9960,10 @@
         <v>1</v>
       </c>
       <c r="F551" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G551" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G551" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="552" spans="1:7" x14ac:dyDescent="0.3">
@@ -9980,10 +9977,10 @@
         <v>1</v>
       </c>
       <c r="F552" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G552" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G552" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="553" spans="1:7" x14ac:dyDescent="0.3">
@@ -10150,10 +10147,10 @@
         <v>1</v>
       </c>
       <c r="F562" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G562" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G562" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="563" spans="1:7" x14ac:dyDescent="0.3">
@@ -10184,10 +10181,10 @@
         <v>1</v>
       </c>
       <c r="F564" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G564" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G564" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="565" spans="1:7" x14ac:dyDescent="0.3">
@@ -10252,10 +10249,10 @@
         <v>1</v>
       </c>
       <c r="F568" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G568" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G568" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="569" spans="1:7" x14ac:dyDescent="0.3">
@@ -10303,10 +10300,10 @@
         <v>1</v>
       </c>
       <c r="F571" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G571" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G571" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="572" spans="1:7" x14ac:dyDescent="0.3">
@@ -10422,10 +10419,10 @@
         <v>1</v>
       </c>
       <c r="F578" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G578" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G578" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="579" spans="1:7" x14ac:dyDescent="0.3">
@@ -10541,10 +10538,10 @@
         <v>1</v>
       </c>
       <c r="F585" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G585" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G585" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="586" spans="1:7" x14ac:dyDescent="0.3">
@@ -10609,10 +10606,10 @@
         <v>1</v>
       </c>
       <c r="F589" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G589" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G589" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="590" spans="1:7" x14ac:dyDescent="0.3">
@@ -10694,10 +10691,10 @@
         <v>1</v>
       </c>
       <c r="F594" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G594" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G594" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="595" spans="1:7" x14ac:dyDescent="0.3">
@@ -10711,10 +10708,10 @@
         <v>1</v>
       </c>
       <c r="F595" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G595" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G595" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="596" spans="1:7" x14ac:dyDescent="0.3">
@@ -10728,10 +10725,10 @@
         <v>1</v>
       </c>
       <c r="F596" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G596" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G596" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="597" spans="1:7" x14ac:dyDescent="0.3">
@@ -11125,10 +11122,10 @@
         <v>1</v>
       </c>
       <c r="F619" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G619" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G619" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="620" spans="1:7" x14ac:dyDescent="0.3">
@@ -11159,10 +11156,10 @@
         <v>1</v>
       </c>
       <c r="F621" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G621" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G621" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="622" spans="1:7" x14ac:dyDescent="0.3">
@@ -11261,10 +11258,10 @@
         <v>1</v>
       </c>
       <c r="F627" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G627" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G627" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="628" spans="1:7" x14ac:dyDescent="0.3">
@@ -11278,10 +11275,10 @@
         <v>1</v>
       </c>
       <c r="F628" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G628" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G628" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="629" spans="1:7" x14ac:dyDescent="0.3">
@@ -11295,10 +11292,10 @@
         <v>1</v>
       </c>
       <c r="F629" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G629" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G629" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="630" spans="1:7" x14ac:dyDescent="0.3">
@@ -11465,10 +11462,10 @@
         <v>1</v>
       </c>
       <c r="F639" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G639" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G639" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="640" spans="1:7" x14ac:dyDescent="0.3">
@@ -11533,10 +11530,10 @@
         <v>1</v>
       </c>
       <c r="F643" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G643" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G643" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="644" spans="1:7" x14ac:dyDescent="0.3">
@@ -11550,10 +11547,10 @@
         <v>1</v>
       </c>
       <c r="F644" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G644" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G644" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="645" spans="1:7" x14ac:dyDescent="0.3">
@@ -11754,10 +11751,10 @@
         <v>1</v>
       </c>
       <c r="F656" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G656" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G656" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="657" spans="1:7" x14ac:dyDescent="0.3">
@@ -11924,10 +11921,10 @@
         <v>1</v>
       </c>
       <c r="F666" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G666" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G666" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="667" spans="1:7" x14ac:dyDescent="0.3">
@@ -12043,10 +12040,10 @@
         <v>1</v>
       </c>
       <c r="F673" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G673" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G673" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="674" spans="1:7" x14ac:dyDescent="0.3">
@@ -12213,10 +12210,10 @@
         <v>1</v>
       </c>
       <c r="F683" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G683" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G683" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="684" spans="1:7" x14ac:dyDescent="0.3">
@@ -12315,10 +12312,10 @@
         <v>1</v>
       </c>
       <c r="F689" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G689" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G689" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="690" spans="1:7" x14ac:dyDescent="0.3">
@@ -12400,10 +12397,10 @@
         <v>1</v>
       </c>
       <c r="F694" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G694" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G694" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="695" spans="1:7" x14ac:dyDescent="0.3">
@@ -12451,10 +12448,10 @@
         <v>1</v>
       </c>
       <c r="F697" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G697" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G697" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="698" spans="1:7" x14ac:dyDescent="0.3">
@@ -12502,10 +12499,10 @@
         <v>1</v>
       </c>
       <c r="F700" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G700" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G700" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="701" spans="1:7" x14ac:dyDescent="0.3">
@@ -12859,10 +12856,10 @@
         <v>1</v>
       </c>
       <c r="F721" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G721" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G721" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="722" spans="1:7" x14ac:dyDescent="0.3">
@@ -12876,10 +12873,10 @@
         <v>1</v>
       </c>
       <c r="F722" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G722" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G722" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="723" spans="1:7" x14ac:dyDescent="0.3">
@@ -12910,10 +12907,10 @@
         <v>1</v>
       </c>
       <c r="F724" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G724" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G724" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="725" spans="1:7" x14ac:dyDescent="0.3">
@@ -12995,10 +12992,10 @@
         <v>1</v>
       </c>
       <c r="F729" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G729" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G729" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="730" spans="1:7" x14ac:dyDescent="0.3">
@@ -13182,10 +13179,10 @@
         <v>1</v>
       </c>
       <c r="F740" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G740" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G740" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="741" spans="1:7" x14ac:dyDescent="0.3">
@@ -13267,10 +13264,10 @@
         <v>1</v>
       </c>
       <c r="F745" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G745" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G745" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="746" spans="1:7" x14ac:dyDescent="0.3">
@@ -13335,10 +13332,10 @@
         <v>1</v>
       </c>
       <c r="F749" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G749" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G749" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="750" spans="1:7" x14ac:dyDescent="0.3">
@@ -13369,10 +13366,10 @@
         <v>1</v>
       </c>
       <c r="F751" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G751" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G751" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="752" spans="1:7" x14ac:dyDescent="0.3">
@@ -13522,10 +13519,10 @@
         <v>1</v>
       </c>
       <c r="F760" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G760" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G760" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="761" spans="1:7" x14ac:dyDescent="0.3">
@@ -13539,10 +13536,10 @@
         <v>1</v>
       </c>
       <c r="F761" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G761" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G761" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="762" spans="1:7" x14ac:dyDescent="0.3">
@@ -13698,10 +13695,10 @@
         <v>1</v>
       </c>
       <c r="F770" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G770" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G770" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="771" spans="1:7" x14ac:dyDescent="0.3">
@@ -13715,10 +13712,10 @@
         <v>1</v>
       </c>
       <c r="F771" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G771" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G771" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="772" spans="1:7" x14ac:dyDescent="0.3">
@@ -13817,10 +13814,10 @@
         <v>1</v>
       </c>
       <c r="F777" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G777" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G777" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="778" spans="1:7" x14ac:dyDescent="0.3">
@@ -13953,10 +13950,10 @@
         <v>1</v>
       </c>
       <c r="F785" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G785" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G785" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="786" spans="1:7" x14ac:dyDescent="0.3">
@@ -14123,10 +14120,10 @@
         <v>1</v>
       </c>
       <c r="F795" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G795" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G795" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="796" spans="1:7" x14ac:dyDescent="0.3">
@@ -14208,10 +14205,10 @@
         <v>1</v>
       </c>
       <c r="F800" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G800" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G800" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="801" spans="1:7" x14ac:dyDescent="0.3">
@@ -14480,10 +14477,10 @@
         <v>1</v>
       </c>
       <c r="F816" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G816" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G816" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="817" spans="1:7" x14ac:dyDescent="0.3">
@@ -14497,10 +14494,10 @@
         <v>1</v>
       </c>
       <c r="F817" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G817" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G817" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="818" spans="1:7" x14ac:dyDescent="0.3">
@@ -14514,10 +14511,10 @@
         <v>1</v>
       </c>
       <c r="F818" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G818" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G818" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="819" spans="1:7" x14ac:dyDescent="0.3">
@@ -14582,10 +14579,10 @@
         <v>1</v>
       </c>
       <c r="F822" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G822" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G822" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="823" spans="1:7" x14ac:dyDescent="0.3">
@@ -14707,10 +14704,10 @@
         <v>1</v>
       </c>
       <c r="F829" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G829" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G829" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="830" spans="1:7" x14ac:dyDescent="0.3">
@@ -14741,10 +14738,10 @@
         <v>1</v>
       </c>
       <c r="F831" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G831" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G831" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="832" spans="1:7" x14ac:dyDescent="0.3">
@@ -14758,10 +14755,10 @@
         <v>1</v>
       </c>
       <c r="F832" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G832" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G832" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="833" spans="1:7" x14ac:dyDescent="0.3">
@@ -14877,10 +14874,10 @@
         <v>1</v>
       </c>
       <c r="F839" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G839" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G839" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="840" spans="1:7" x14ac:dyDescent="0.3">
@@ -14911,10 +14908,10 @@
         <v>1</v>
       </c>
       <c r="F841" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G841" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G841" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="842" spans="1:7" x14ac:dyDescent="0.3">
@@ -14928,10 +14925,10 @@
         <v>1</v>
       </c>
       <c r="F842" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G842" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G842" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="843" spans="1:7" x14ac:dyDescent="0.3">
@@ -15064,10 +15061,10 @@
         <v>1</v>
       </c>
       <c r="F850" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G850" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G850" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="851" spans="1:7" x14ac:dyDescent="0.3">
@@ -15115,10 +15112,10 @@
         <v>1</v>
       </c>
       <c r="F853" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G853" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G853" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="854" spans="1:7" x14ac:dyDescent="0.3">
@@ -15149,10 +15146,10 @@
         <v>1</v>
       </c>
       <c r="F855" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G855" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G855" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="856" spans="1:7" x14ac:dyDescent="0.3">
@@ -15166,10 +15163,10 @@
         <v>1</v>
       </c>
       <c r="F856" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G856" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G856" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="857" spans="1:7" x14ac:dyDescent="0.3">
@@ -15274,10 +15271,10 @@
         <v>1</v>
       </c>
       <c r="F862" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G862" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G862" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="863" spans="1:7" x14ac:dyDescent="0.3">
@@ -15512,10 +15509,10 @@
         <v>1</v>
       </c>
       <c r="F876" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G876" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G876" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="877" spans="1:7" x14ac:dyDescent="0.3">
@@ -15597,10 +15594,10 @@
         <v>1</v>
       </c>
       <c r="F881" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G881" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G881" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="882" spans="1:7" x14ac:dyDescent="0.3">
@@ -15665,10 +15662,10 @@
         <v>1</v>
       </c>
       <c r="F885" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G885" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G885" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="886" spans="1:7" x14ac:dyDescent="0.3">
@@ -15835,10 +15832,10 @@
         <v>1</v>
       </c>
       <c r="F895" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G895" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G895" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="896" spans="1:7" x14ac:dyDescent="0.3">
@@ -16056,10 +16053,10 @@
         <v>1</v>
       </c>
       <c r="F908" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G908" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G908" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="909" spans="1:7" x14ac:dyDescent="0.3">
@@ -16147,10 +16144,10 @@
         <v>1</v>
       </c>
       <c r="F913" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G913" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G913" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="914" spans="1:7" x14ac:dyDescent="0.3">
@@ -16215,10 +16212,10 @@
         <v>1</v>
       </c>
       <c r="F917" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G917" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G917" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="918" spans="1:7" x14ac:dyDescent="0.3">
@@ -16368,10 +16365,10 @@
         <v>1</v>
       </c>
       <c r="F926" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G926" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G926" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="927" spans="1:7" x14ac:dyDescent="0.3">
@@ -16436,10 +16433,10 @@
         <v>1</v>
       </c>
       <c r="F930" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G930" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G930" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="931" spans="1:7" x14ac:dyDescent="0.3">
@@ -16487,10 +16484,10 @@
         <v>1</v>
       </c>
       <c r="F933" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G933" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G933" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="934" spans="1:7" x14ac:dyDescent="0.3">
@@ -16589,10 +16586,10 @@
         <v>1</v>
       </c>
       <c r="F939" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G939" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G939" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="940" spans="1:7" x14ac:dyDescent="0.3">
@@ -16674,10 +16671,10 @@
         <v>1</v>
       </c>
       <c r="F944" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G944" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G944" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="945" spans="1:7" x14ac:dyDescent="0.3">
@@ -16912,10 +16909,10 @@
         <v>1</v>
       </c>
       <c r="F958" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G958" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G958" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="959" spans="1:7" x14ac:dyDescent="0.3">
@@ -16963,10 +16960,10 @@
         <v>1</v>
       </c>
       <c r="F961" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G961" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G961" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="962" spans="1:7" x14ac:dyDescent="0.3">
@@ -17031,10 +17028,10 @@
         <v>1</v>
       </c>
       <c r="F965" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G965" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G965" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="966" spans="1:7" x14ac:dyDescent="0.3">
@@ -17439,10 +17436,10 @@
         <v>1</v>
       </c>
       <c r="F989" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G989" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G989" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="990" spans="1:7" x14ac:dyDescent="0.3">
@@ -17473,10 +17470,10 @@
         <v>1</v>
       </c>
       <c r="F991" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G991" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G991" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="992" spans="1:7" x14ac:dyDescent="0.3">
@@ -17626,10 +17623,10 @@
         <v>1</v>
       </c>
       <c r="F1000" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1000" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1000" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1001" spans="1:7" x14ac:dyDescent="0.3">
@@ -17660,10 +17657,10 @@
         <v>1</v>
       </c>
       <c r="F1002" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1002" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1002" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1003" spans="1:7" x14ac:dyDescent="0.3">
@@ -17751,10 +17748,10 @@
         <v>1</v>
       </c>
       <c r="F1007" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1007" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1007" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1008" spans="1:7" x14ac:dyDescent="0.3">
@@ -17768,10 +17765,10 @@
         <v>1</v>
       </c>
       <c r="F1008" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1008" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1008" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1009" spans="1:7" x14ac:dyDescent="0.3">
@@ -17802,10 +17799,10 @@
         <v>1</v>
       </c>
       <c r="F1010" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1010" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1010" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1011" spans="1:7" x14ac:dyDescent="0.3">
@@ -18295,10 +18292,10 @@
         <v>1</v>
       </c>
       <c r="F1039" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1039" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1039" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1040" spans="1:7" x14ac:dyDescent="0.3">
@@ -18499,10 +18496,10 @@
         <v>1</v>
       </c>
       <c r="F1051" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1051" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1051" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1052" spans="1:7" x14ac:dyDescent="0.3">
@@ -18601,10 +18598,10 @@
         <v>1</v>
       </c>
       <c r="F1057" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1057" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1057" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1058" spans="1:7" x14ac:dyDescent="0.3">
@@ -18771,10 +18768,10 @@
         <v>1</v>
       </c>
       <c r="F1067" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1067" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1067" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1068" spans="1:7" x14ac:dyDescent="0.3">
@@ -19145,10 +19142,10 @@
         <v>1</v>
       </c>
       <c r="F1089" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1089" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1089" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1090" spans="1:7" x14ac:dyDescent="0.3">
@@ -19247,10 +19244,10 @@
         <v>1</v>
       </c>
       <c r="F1095" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1095" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1095" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1096" spans="1:7" x14ac:dyDescent="0.3">
@@ -19281,10 +19278,10 @@
         <v>1</v>
       </c>
       <c r="F1097" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1097" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1097" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1098" spans="1:7" x14ac:dyDescent="0.3">
@@ -19332,10 +19329,10 @@
         <v>1</v>
       </c>
       <c r="F1100" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1100" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1100" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1101" spans="1:7" x14ac:dyDescent="0.3">
@@ -19383,10 +19380,10 @@
         <v>1</v>
       </c>
       <c r="F1103" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1103" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1103" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1104" spans="1:7" x14ac:dyDescent="0.3">
@@ -19485,10 +19482,10 @@
         <v>1</v>
       </c>
       <c r="F1109" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1109" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1109" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1110" spans="1:7" x14ac:dyDescent="0.3">
@@ -19655,10 +19652,10 @@
         <v>1</v>
       </c>
       <c r="F1119" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1119" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1119" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1120" spans="1:7" x14ac:dyDescent="0.3">
@@ -19689,10 +19686,10 @@
         <v>1</v>
       </c>
       <c r="F1121" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1121" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1121" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1122" spans="1:7" x14ac:dyDescent="0.3">
@@ -19757,10 +19754,10 @@
         <v>1</v>
       </c>
       <c r="F1125" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1125" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1125" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1126" spans="1:7" x14ac:dyDescent="0.3">
@@ -19808,10 +19805,10 @@
         <v>1</v>
       </c>
       <c r="F1128" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1128" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1128" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1129" spans="1:7" x14ac:dyDescent="0.3">
@@ -20012,10 +20009,10 @@
         <v>1</v>
       </c>
       <c r="F1140" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1140" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1140" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1141" spans="1:7" x14ac:dyDescent="0.3">
@@ -20114,10 +20111,10 @@
         <v>1</v>
       </c>
       <c r="F1146" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1146" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1146" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1147" spans="1:7" x14ac:dyDescent="0.3">
@@ -20131,10 +20128,10 @@
         <v>1</v>
       </c>
       <c r="F1147" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1147" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1147" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1148" spans="1:7" x14ac:dyDescent="0.3">
@@ -20250,10 +20247,10 @@
         <v>1</v>
       </c>
       <c r="F1154" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1154" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1154" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1155" spans="1:7" x14ac:dyDescent="0.3">
@@ -20318,10 +20315,10 @@
         <v>1</v>
       </c>
       <c r="F1158" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1158" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1158" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1159" spans="1:7" x14ac:dyDescent="0.3">
@@ -20369,10 +20366,10 @@
         <v>1</v>
       </c>
       <c r="F1161" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1161" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1161" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1162" spans="1:7" x14ac:dyDescent="0.3">
@@ -20454,10 +20451,10 @@
         <v>1</v>
       </c>
       <c r="F1166" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1166" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1166" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1167" spans="1:7" x14ac:dyDescent="0.3">
@@ -20658,10 +20655,10 @@
         <v>1</v>
       </c>
       <c r="F1178" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1178" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1178" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1179" spans="1:7" x14ac:dyDescent="0.3">
@@ -20709,10 +20706,10 @@
         <v>1</v>
       </c>
       <c r="F1181" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1181" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1181" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1182" spans="1:7" x14ac:dyDescent="0.3">
@@ -20743,10 +20740,10 @@
         <v>1</v>
       </c>
       <c r="F1183" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1183" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1183" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1184" spans="1:7" x14ac:dyDescent="0.3">
@@ -20828,10 +20825,10 @@
         <v>1</v>
       </c>
       <c r="F1188" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1188" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1188" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1189" spans="1:7" x14ac:dyDescent="0.3">
@@ -20947,10 +20944,10 @@
         <v>1</v>
       </c>
       <c r="F1195" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1195" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1195" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1196" spans="1:7" x14ac:dyDescent="0.3">
@@ -20981,10 +20978,10 @@
         <v>1</v>
       </c>
       <c r="F1197" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1197" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1197" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1198" spans="1:7" x14ac:dyDescent="0.3">
@@ -21049,10 +21046,10 @@
         <v>1</v>
       </c>
       <c r="F1201" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1201" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1201" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1202" spans="1:7" x14ac:dyDescent="0.3">
@@ -21066,10 +21063,10 @@
         <v>1</v>
       </c>
       <c r="F1202" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1202" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1202" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1203" spans="1:7" x14ac:dyDescent="0.3">
@@ -21100,10 +21097,10 @@
         <v>1</v>
       </c>
       <c r="F1204" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1204" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1204" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1205" spans="1:7" x14ac:dyDescent="0.3">
@@ -21151,10 +21148,10 @@
         <v>1</v>
       </c>
       <c r="F1207" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1207" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1207" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1208" spans="1:7" x14ac:dyDescent="0.3">
@@ -21293,10 +21290,10 @@
         <v>1</v>
       </c>
       <c r="F1215" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1215" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1215" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1216" spans="1:7" x14ac:dyDescent="0.3">
@@ -21327,10 +21324,10 @@
         <v>1</v>
       </c>
       <c r="F1217" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1217" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1217" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1218" spans="1:7" x14ac:dyDescent="0.3">
@@ -21344,10 +21341,10 @@
         <v>1</v>
       </c>
       <c r="F1218" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1218" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1218" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1219" spans="1:7" x14ac:dyDescent="0.3">
@@ -21429,10 +21426,10 @@
         <v>1</v>
       </c>
       <c r="F1223" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1223" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1223" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1224" spans="1:7" x14ac:dyDescent="0.3">
@@ -21741,10 +21738,10 @@
         <v>1</v>
       </c>
       <c r="F1241" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1241" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1241" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1242" spans="1:7" x14ac:dyDescent="0.3">
@@ -21758,10 +21755,10 @@
         <v>1</v>
       </c>
       <c r="F1242" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1242" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1242" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1243" spans="1:7" x14ac:dyDescent="0.3">
@@ -21826,10 +21823,10 @@
         <v>1</v>
       </c>
       <c r="F1246" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1246" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1246" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1247" spans="1:7" x14ac:dyDescent="0.3">
@@ -21928,10 +21925,10 @@
         <v>1</v>
       </c>
       <c r="F1252" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1252" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1252" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1253" spans="1:7" x14ac:dyDescent="0.3">
@@ -22047,10 +22044,10 @@
         <v>1</v>
       </c>
       <c r="F1259" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1259" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1259" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1260" spans="1:7" x14ac:dyDescent="0.3">
@@ -22098,10 +22095,10 @@
         <v>1</v>
       </c>
       <c r="F1262" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1262" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1262" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1263" spans="1:7" x14ac:dyDescent="0.3">
@@ -22166,10 +22163,10 @@
         <v>1</v>
       </c>
       <c r="F1266" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1266" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1266" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1267" spans="1:7" x14ac:dyDescent="0.3">
@@ -22268,10 +22265,10 @@
         <v>1</v>
       </c>
       <c r="F1272" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1272" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1272" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1273" spans="1:7" x14ac:dyDescent="0.3">
@@ -22285,10 +22282,10 @@
         <v>1</v>
       </c>
       <c r="F1273" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1273" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1273" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1274" spans="1:7" x14ac:dyDescent="0.3">
@@ -22353,10 +22350,10 @@
         <v>1</v>
       </c>
       <c r="F1277" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1277" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1277" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1278" spans="1:7" x14ac:dyDescent="0.3">
@@ -22438,10 +22435,10 @@
         <v>1</v>
       </c>
       <c r="F1282" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1282" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1282" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1283" spans="1:7" x14ac:dyDescent="0.3">
@@ -22540,10 +22537,10 @@
         <v>1</v>
       </c>
       <c r="F1288" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1288" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1288" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1289" spans="1:7" x14ac:dyDescent="0.3">
@@ -22710,10 +22707,10 @@
         <v>1</v>
       </c>
       <c r="F1298" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1298" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1298" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1299" spans="1:7" x14ac:dyDescent="0.3">
@@ -22727,10 +22724,10 @@
         <v>1</v>
       </c>
       <c r="F1299" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1299" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1299" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1300" spans="1:7" x14ac:dyDescent="0.3">
@@ -22767,10 +22764,10 @@
         <v>1</v>
       </c>
       <c r="F1301" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1301" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1301" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1302" spans="1:7" x14ac:dyDescent="0.3">
@@ -22983,10 +22980,10 @@
         <v>1</v>
       </c>
       <c r="F1313" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1313" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1313" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1314" spans="1:7" x14ac:dyDescent="0.3">
@@ -23068,10 +23065,10 @@
         <v>1</v>
       </c>
       <c r="F1318" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1318" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1318" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1319" spans="1:7" x14ac:dyDescent="0.3">
@@ -23204,10 +23201,10 @@
         <v>1</v>
       </c>
       <c r="F1326" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1326" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1326" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1327" spans="1:7" x14ac:dyDescent="0.3">
@@ -23221,10 +23218,10 @@
         <v>1</v>
       </c>
       <c r="F1327" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1327" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1327" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1328" spans="1:7" x14ac:dyDescent="0.3">
@@ -23323,10 +23320,10 @@
         <v>1</v>
       </c>
       <c r="F1333" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1333" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1333" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1334" spans="1:7" x14ac:dyDescent="0.3">
@@ -23374,10 +23371,10 @@
         <v>1</v>
       </c>
       <c r="F1336" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1336" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1336" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1337" spans="1:7" x14ac:dyDescent="0.3">
@@ -23391,10 +23388,10 @@
         <v>1</v>
       </c>
       <c r="F1337" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1337" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1337" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1338" spans="1:7" x14ac:dyDescent="0.3">
@@ -23442,10 +23439,10 @@
         <v>1</v>
       </c>
       <c r="F1340" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1340" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1340" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1341" spans="1:7" x14ac:dyDescent="0.3">
@@ -23459,10 +23456,10 @@
         <v>1</v>
       </c>
       <c r="F1341" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1341" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1341" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1342" spans="1:7" x14ac:dyDescent="0.3">
@@ -23561,10 +23558,10 @@
         <v>1</v>
       </c>
       <c r="F1347" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1347" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1347" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1348" spans="1:7" x14ac:dyDescent="0.3">
@@ -23629,10 +23626,10 @@
         <v>1</v>
       </c>
       <c r="F1351" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1351" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1351" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1352" spans="1:7" x14ac:dyDescent="0.3">
@@ -23697,10 +23694,10 @@
         <v>1</v>
       </c>
       <c r="F1355" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1355" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1355" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1356" spans="1:7" x14ac:dyDescent="0.3">
@@ -23799,10 +23796,10 @@
         <v>1</v>
       </c>
       <c r="F1361" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1361" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1361" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1362" spans="1:7" x14ac:dyDescent="0.3">
@@ -23816,10 +23813,10 @@
         <v>1</v>
       </c>
       <c r="F1362" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1362" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1362" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1363" spans="1:7" x14ac:dyDescent="0.3">
@@ -23867,10 +23864,10 @@
         <v>1</v>
       </c>
       <c r="F1365" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1365" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1365" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1366" spans="1:7" x14ac:dyDescent="0.3">
@@ -23952,10 +23949,10 @@
         <v>1</v>
       </c>
       <c r="F1370" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1370" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1370" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1371" spans="1:7" x14ac:dyDescent="0.3">
@@ -24111,10 +24108,10 @@
         <v>1</v>
       </c>
       <c r="F1379" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1379" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1379" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1380" spans="1:7" x14ac:dyDescent="0.3">
@@ -24145,10 +24142,10 @@
         <v>1</v>
       </c>
       <c r="F1381" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1381" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1381" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1382" spans="1:7" x14ac:dyDescent="0.3">
@@ -24179,10 +24176,10 @@
         <v>1</v>
       </c>
       <c r="F1383" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1383" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1383" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1384" spans="1:7" x14ac:dyDescent="0.3">
@@ -24213,10 +24210,10 @@
         <v>1</v>
       </c>
       <c r="F1385" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1385" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1385" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1386" spans="1:7" x14ac:dyDescent="0.3">
@@ -24264,10 +24261,10 @@
         <v>1</v>
       </c>
       <c r="F1388" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1388" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1388" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1389" spans="1:7" x14ac:dyDescent="0.3">
@@ -24349,10 +24346,10 @@
         <v>1</v>
       </c>
       <c r="F1393" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1393" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1393" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1394" spans="1:7" x14ac:dyDescent="0.3">
@@ -24366,10 +24363,10 @@
         <v>1</v>
       </c>
       <c r="F1394" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1394" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1394" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1395" spans="1:7" x14ac:dyDescent="0.3">
@@ -24468,10 +24465,10 @@
         <v>1</v>
       </c>
       <c r="F1400" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1400" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1400" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1401" spans="1:7" x14ac:dyDescent="0.3">
@@ -24519,10 +24516,10 @@
         <v>1</v>
       </c>
       <c r="F1403" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1403" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1403" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1404" spans="1:7" x14ac:dyDescent="0.3">
@@ -24587,10 +24584,10 @@
         <v>1</v>
       </c>
       <c r="F1407" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1407" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1407" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1408" spans="1:7" x14ac:dyDescent="0.3">
@@ -24621,10 +24618,10 @@
         <v>1</v>
       </c>
       <c r="F1409" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1409" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1409" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1410" spans="1:7" x14ac:dyDescent="0.3">
@@ -24678,10 +24675,10 @@
         <v>1</v>
       </c>
       <c r="F1412" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1412" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1412" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1413" spans="1:7" x14ac:dyDescent="0.3">
@@ -24695,10 +24692,10 @@
         <v>1</v>
       </c>
       <c r="F1413" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1413" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1413" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1414" spans="1:7" x14ac:dyDescent="0.3">
@@ -24712,10 +24709,10 @@
         <v>1</v>
       </c>
       <c r="F1414" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1414" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1414" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1415" spans="1:7" x14ac:dyDescent="0.3">
@@ -24729,10 +24726,10 @@
         <v>1</v>
       </c>
       <c r="F1415" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1415" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1415" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1416" spans="1:7" x14ac:dyDescent="0.3">
@@ -24746,10 +24743,10 @@
         <v>1</v>
       </c>
       <c r="F1416" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1416" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1416" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1417" spans="1:7" x14ac:dyDescent="0.3">
@@ -24814,10 +24811,10 @@
         <v>1</v>
       </c>
       <c r="F1420" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1420" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1420" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1421" spans="1:7" x14ac:dyDescent="0.3">
@@ -24882,10 +24879,10 @@
         <v>1</v>
       </c>
       <c r="F1424" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1424" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1424" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1425" spans="1:7" x14ac:dyDescent="0.3">
@@ -24916,10 +24913,10 @@
         <v>1</v>
       </c>
       <c r="F1426" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1426" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1426" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1427" spans="1:7" x14ac:dyDescent="0.3">
@@ -24956,10 +24953,10 @@
         <v>1</v>
       </c>
       <c r="F1428" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1428" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1428" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1429" spans="1:7" x14ac:dyDescent="0.3">
@@ -25047,10 +25044,10 @@
         <v>1</v>
       </c>
       <c r="F1433" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1433" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1433" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1434" spans="1:7" x14ac:dyDescent="0.3">
@@ -25115,10 +25112,10 @@
         <v>1</v>
       </c>
       <c r="F1437" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1437" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1437" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1438" spans="1:7" x14ac:dyDescent="0.3">
@@ -25132,10 +25129,10 @@
         <v>1</v>
       </c>
       <c r="F1438" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1438" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1438" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1439" spans="1:7" x14ac:dyDescent="0.3">
@@ -25268,10 +25265,10 @@
         <v>1</v>
       </c>
       <c r="F1446" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1446" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1446" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1447" spans="1:7" x14ac:dyDescent="0.3">
@@ -25285,10 +25282,10 @@
         <v>1</v>
       </c>
       <c r="F1447" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1447" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1447" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1448" spans="1:7" x14ac:dyDescent="0.3">
@@ -25302,10 +25299,10 @@
         <v>1</v>
       </c>
       <c r="F1448" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1448" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1448" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1449" spans="1:7" x14ac:dyDescent="0.3">
@@ -25336,10 +25333,10 @@
         <v>1</v>
       </c>
       <c r="F1450" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1450" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1450" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1451" spans="1:7" x14ac:dyDescent="0.3">
@@ -25353,10 +25350,10 @@
         <v>1</v>
       </c>
       <c r="F1451" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1451" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1451" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1452" spans="1:7" x14ac:dyDescent="0.3">
@@ -25370,10 +25367,10 @@
         <v>1</v>
       </c>
       <c r="F1452" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1452" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1452" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1453" spans="1:7" x14ac:dyDescent="0.3">
@@ -25387,10 +25384,10 @@
         <v>1</v>
       </c>
       <c r="F1453" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1453" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1453" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1454" spans="1:7" x14ac:dyDescent="0.3">
@@ -25404,10 +25401,10 @@
         <v>1</v>
       </c>
       <c r="F1454" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1454" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1454" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1455" spans="1:7" x14ac:dyDescent="0.3">
@@ -25438,10 +25435,10 @@
         <v>1</v>
       </c>
       <c r="F1456" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1456" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1456" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1457" spans="1:7" x14ac:dyDescent="0.3">
@@ -25472,10 +25469,10 @@
         <v>1</v>
       </c>
       <c r="F1458" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1458" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1458" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1459" spans="1:7" x14ac:dyDescent="0.3">
@@ -25489,10 +25486,10 @@
         <v>1</v>
       </c>
       <c r="F1459" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1459" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1459" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1460" spans="1:7" x14ac:dyDescent="0.3">
@@ -25506,10 +25503,10 @@
         <v>1</v>
       </c>
       <c r="F1460" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1460" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1460" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1461" spans="1:7" x14ac:dyDescent="0.3">
@@ -25614,10 +25611,10 @@
         <v>1</v>
       </c>
       <c r="F1466" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1466" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1466" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1467" spans="1:7" x14ac:dyDescent="0.3">
@@ -25648,10 +25645,10 @@
         <v>1</v>
       </c>
       <c r="F1468" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1468" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1468" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1469" spans="1:7" x14ac:dyDescent="0.3">
@@ -25722,10 +25719,10 @@
         <v>1</v>
       </c>
       <c r="F1472" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1472" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1472" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1473" spans="1:7" x14ac:dyDescent="0.3">
@@ -25807,10 +25804,10 @@
         <v>1</v>
       </c>
       <c r="F1477" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1477" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1477" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1478" spans="1:7" x14ac:dyDescent="0.3">
@@ -25915,10 +25912,10 @@
         <v>1</v>
       </c>
       <c r="F1483" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1483" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1483" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1484" spans="1:7" x14ac:dyDescent="0.3">
@@ -26017,10 +26014,10 @@
         <v>1</v>
       </c>
       <c r="F1489" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1489" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1489" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1490" spans="1:7" x14ac:dyDescent="0.3">
@@ -26068,10 +26065,10 @@
         <v>1</v>
       </c>
       <c r="F1492" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1492" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1492" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1493" spans="1:7" x14ac:dyDescent="0.3">
@@ -26159,10 +26156,10 @@
         <v>1</v>
       </c>
       <c r="F1497" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1497" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1497" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1498" spans="1:7" x14ac:dyDescent="0.3">
@@ -26176,10 +26173,10 @@
         <v>1</v>
       </c>
       <c r="F1498" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1498" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1498" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1499" spans="1:7" x14ac:dyDescent="0.3">
@@ -26216,10 +26213,10 @@
         <v>1</v>
       </c>
       <c r="F1500" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1500" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1500" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1501" spans="1:7" x14ac:dyDescent="0.3">
@@ -26267,10 +26264,10 @@
         <v>1</v>
       </c>
       <c r="F1503" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1503" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1503" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1504" spans="1:7" x14ac:dyDescent="0.3">
@@ -26335,10 +26332,10 @@
         <v>1</v>
       </c>
       <c r="F1507" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1507" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1507" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1508" spans="1:7" x14ac:dyDescent="0.3">
@@ -26369,10 +26366,10 @@
         <v>1</v>
       </c>
       <c r="F1509" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1509" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1509" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1510" spans="1:7" x14ac:dyDescent="0.3">
@@ -26403,10 +26400,10 @@
         <v>1</v>
       </c>
       <c r="F1511" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1511" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1511" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1512" spans="1:7" x14ac:dyDescent="0.3">
@@ -26420,10 +26417,10 @@
         <v>1</v>
       </c>
       <c r="F1512" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1512" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1512" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1513" spans="1:7" x14ac:dyDescent="0.3">
@@ -26488,10 +26485,10 @@
         <v>1</v>
       </c>
       <c r="F1516" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1516" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1516" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1517" spans="1:7" x14ac:dyDescent="0.3">
@@ -26556,10 +26553,10 @@
         <v>1</v>
       </c>
       <c r="F1520" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1520" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1520" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1521" spans="1:7" x14ac:dyDescent="0.3">
@@ -26607,10 +26604,10 @@
         <v>1</v>
       </c>
       <c r="F1523" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1523" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1523" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1524" spans="1:7" x14ac:dyDescent="0.3">
@@ -26726,10 +26723,10 @@
         <v>1</v>
       </c>
       <c r="F1530" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1530" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1530" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1531" spans="1:7" x14ac:dyDescent="0.3">
@@ -26743,10 +26740,10 @@
         <v>1</v>
       </c>
       <c r="F1531" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1531" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1531" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1532" spans="1:7" x14ac:dyDescent="0.3">
@@ -26811,10 +26808,10 @@
         <v>1</v>
       </c>
       <c r="F1535" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1535" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1535" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1536" spans="1:7" x14ac:dyDescent="0.3">
@@ -26828,10 +26825,10 @@
         <v>1</v>
       </c>
       <c r="F1536" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1536" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1536" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1537" spans="1:7" x14ac:dyDescent="0.3">
@@ -26862,10 +26859,10 @@
         <v>1</v>
       </c>
       <c r="F1538" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1538" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1538" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1539" spans="1:7" x14ac:dyDescent="0.3">
@@ -26896,10 +26893,10 @@
         <v>1</v>
       </c>
       <c r="F1540" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1540" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1540" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1541" spans="1:7" x14ac:dyDescent="0.3">
@@ -26930,10 +26927,10 @@
         <v>1</v>
       </c>
       <c r="F1542" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1542" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1542" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1543" spans="1:7" x14ac:dyDescent="0.3">
@@ -26981,10 +26978,10 @@
         <v>1</v>
       </c>
       <c r="F1545" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1545" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1545" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1546" spans="1:7" x14ac:dyDescent="0.3">
@@ -26998,10 +26995,10 @@
         <v>1</v>
       </c>
       <c r="F1546" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1546" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1546" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1547" spans="1:7" x14ac:dyDescent="0.3">
@@ -27015,10 +27012,10 @@
         <v>1</v>
       </c>
       <c r="F1547" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1547" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1547" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1548" spans="1:7" x14ac:dyDescent="0.3">
@@ -27049,10 +27046,10 @@
         <v>1</v>
       </c>
       <c r="F1549" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1549" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1549" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1550" spans="1:7" x14ac:dyDescent="0.3">
@@ -27134,10 +27131,10 @@
         <v>1</v>
       </c>
       <c r="F1554" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1554" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1554" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1555" spans="1:7" x14ac:dyDescent="0.3">
@@ -27219,10 +27216,10 @@
         <v>1</v>
       </c>
       <c r="F1559" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1559" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1559" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1560" spans="1:7" x14ac:dyDescent="0.3">
@@ -27270,10 +27267,10 @@
         <v>1</v>
       </c>
       <c r="F1562" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1562" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1562" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1563" spans="1:7" x14ac:dyDescent="0.3">
@@ -27304,10 +27301,10 @@
         <v>1</v>
       </c>
       <c r="F1564" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1564" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1564" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1565" spans="1:7" x14ac:dyDescent="0.3">
@@ -27321,10 +27318,10 @@
         <v>1</v>
       </c>
       <c r="F1565" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1565" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1565" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1566" spans="1:7" x14ac:dyDescent="0.3">
@@ -27463,10 +27460,10 @@
         <v>1</v>
       </c>
       <c r="F1573" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1573" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1573" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1574" spans="1:7" x14ac:dyDescent="0.3">
@@ -27514,10 +27511,10 @@
         <v>1</v>
       </c>
       <c r="F1576" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1576" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1576" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1577" spans="1:7" x14ac:dyDescent="0.3">
@@ -27650,10 +27647,10 @@
         <v>1</v>
       </c>
       <c r="F1584" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1584" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1584" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1585" spans="1:7" x14ac:dyDescent="0.3">
@@ -27684,10 +27681,10 @@
         <v>1</v>
       </c>
       <c r="F1586" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1586" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1586" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1587" spans="1:7" x14ac:dyDescent="0.3">
@@ -27718,10 +27715,10 @@
         <v>1</v>
       </c>
       <c r="F1588" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1588" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1588" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1589" spans="1:7" x14ac:dyDescent="0.3">
@@ -27735,10 +27732,10 @@
         <v>1</v>
       </c>
       <c r="F1589" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1589" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1589" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1590" spans="1:7" x14ac:dyDescent="0.3">
@@ -27752,10 +27749,10 @@
         <v>1</v>
       </c>
       <c r="F1590" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1590" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1590" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1591" spans="1:7" x14ac:dyDescent="0.3">
@@ -27786,10 +27783,10 @@
         <v>1</v>
       </c>
       <c r="F1592" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1592" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1592" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1593" spans="1:7" x14ac:dyDescent="0.3">
@@ -27888,10 +27885,10 @@
         <v>1</v>
       </c>
       <c r="F1598" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1598" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1598" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1599" spans="1:7" x14ac:dyDescent="0.3">
@@ -27905,10 +27902,10 @@
         <v>1</v>
       </c>
       <c r="F1599" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1599" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1599" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1600" spans="1:7" x14ac:dyDescent="0.3">
@@ -27973,10 +27970,10 @@
         <v>1</v>
       </c>
       <c r="F1603" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1603" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1603" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1604" spans="1:7" x14ac:dyDescent="0.3">
@@ -28024,10 +28021,10 @@
         <v>1</v>
       </c>
       <c r="F1606" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1606" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1606" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1607" spans="1:7" x14ac:dyDescent="0.3">
@@ -28041,10 +28038,10 @@
         <v>1</v>
       </c>
       <c r="F1607" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1607" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1607" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1608" spans="1:7" x14ac:dyDescent="0.3">
@@ -28058,10 +28055,10 @@
         <v>1</v>
       </c>
       <c r="F1608" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1608" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1608" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1609" spans="1:7" x14ac:dyDescent="0.3">
@@ -28109,10 +28106,10 @@
         <v>1</v>
       </c>
       <c r="F1611" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1611" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1611" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1612" spans="1:7" x14ac:dyDescent="0.3">
@@ -28126,10 +28123,10 @@
         <v>1</v>
       </c>
       <c r="F1612" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1612" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1612" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1613" spans="1:7" x14ac:dyDescent="0.3">
@@ -28143,10 +28140,10 @@
         <v>1</v>
       </c>
       <c r="F1613" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1613" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1613" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1614" spans="1:7" x14ac:dyDescent="0.3">
@@ -28228,10 +28225,10 @@
         <v>1</v>
       </c>
       <c r="F1618" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1618" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1618" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1619" spans="1:7" x14ac:dyDescent="0.3">
@@ -28296,10 +28293,10 @@
         <v>1</v>
       </c>
       <c r="F1622" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1622" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1622" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1623" spans="1:7" x14ac:dyDescent="0.3">
@@ -28313,10 +28310,10 @@
         <v>1</v>
       </c>
       <c r="F1623" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1623" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1623" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1624" spans="1:7" x14ac:dyDescent="0.3">
@@ -28500,10 +28497,10 @@
         <v>1</v>
       </c>
       <c r="F1634" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1634" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1634" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1635" spans="1:7" x14ac:dyDescent="0.3">
@@ -28534,10 +28531,10 @@
         <v>1</v>
       </c>
       <c r="F1636" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1636" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1636" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1637" spans="1:7" x14ac:dyDescent="0.3">
@@ -28585,10 +28582,10 @@
         <v>1</v>
       </c>
       <c r="F1639" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1639" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1639" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1640" spans="1:7" x14ac:dyDescent="0.3">
@@ -28670,10 +28667,10 @@
         <v>1</v>
       </c>
       <c r="F1644" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1644" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1644" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1645" spans="1:7" x14ac:dyDescent="0.3">
@@ -28721,10 +28718,10 @@
         <v>1</v>
       </c>
       <c r="F1647" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1647" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1647" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1648" spans="1:7" x14ac:dyDescent="0.3">
@@ -28772,10 +28769,10 @@
         <v>1</v>
       </c>
       <c r="F1650" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1650" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1650" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1651" spans="1:7" x14ac:dyDescent="0.3">
@@ -28857,10 +28854,10 @@
         <v>1</v>
       </c>
       <c r="F1655" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1655" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1655" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1656" spans="1:7" x14ac:dyDescent="0.3">
@@ -28908,10 +28905,10 @@
         <v>1</v>
       </c>
       <c r="F1658" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1658" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1658" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1659" spans="1:7" x14ac:dyDescent="0.3">
@@ -28976,10 +28973,10 @@
         <v>1</v>
       </c>
       <c r="F1662" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1662" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1662" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1663" spans="1:7" x14ac:dyDescent="0.3">
@@ -29163,10 +29160,10 @@
         <v>1</v>
       </c>
       <c r="F1673" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1673" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1673" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1674" spans="1:7" x14ac:dyDescent="0.3">
@@ -29316,10 +29313,10 @@
         <v>1</v>
       </c>
       <c r="F1682" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1682" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G1682" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="1683" spans="1:7" x14ac:dyDescent="0.3">

</xml_diff>